<commit_message>
feat: edicion de planillas de busqueda en la app
- Las 3 planillas (colores AUTOPAK, colores BYD, modelos Nissan) se muestran
  como tarjetas con su cantidad cargada.
- "Ver y editar" abre la planilla en un panel con tabla editable: buscar,
  modificar, agregar y borrar filas; marca celdas modificadas, filas nuevas,
  codigos repetidos y filas incompletas, y guarda la planilla completa (PUT).
- Descarga de cada planilla tal como esta cargada (mismo orden y formato que
  se puede volver a subir) y reemplazo por .xlsx.
- Las subidas se leen desde un temporal en vez de copiarse a lookup_tables/,
  y una planilla vacia o invalida se rechaza sin tocar la cargada.
- Planillas semilla actualizadas a las versiones cargadas el 08/10/2026.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/lookup_tables/codigos de colores byd.xlsx
+++ b/server/lookup_tables/codigos de colores byd.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gactis\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lisandro Santori\Documents\Neostar\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20340" windowHeight="6990"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20340" windowHeight="6996"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
   <si>
     <t>Código</t>
   </si>
@@ -32,15 +32,9 @@
     <t>Descripción</t>
   </si>
   <si>
-    <t xml:space="preserve">BYD06 </t>
-  </si>
-  <si>
     <t>APRICITY WHITE/BLACK&amp;GRAY DUAL</t>
   </si>
   <si>
-    <t xml:space="preserve">DYB07 </t>
-  </si>
-  <si>
     <t xml:space="preserve">ATLANTIS BLUE                 </t>
   </si>
   <si>
@@ -56,45 +50,24 @@
     <t xml:space="preserve">ATLANTIS BLUE/GRAVEL BEIGE    </t>
   </si>
   <si>
-    <t xml:space="preserve">AGB   </t>
-  </si>
-  <si>
     <t xml:space="preserve">ATLANTIS GREY/BLACK           </t>
   </si>
   <si>
-    <t xml:space="preserve">BYD01 </t>
-  </si>
-  <si>
     <t xml:space="preserve">BLACK SKIING WHITE            </t>
   </si>
   <si>
-    <t xml:space="preserve">BYD04 </t>
-  </si>
-  <si>
     <t xml:space="preserve">BLACK SNOW  WHITE             </t>
   </si>
   <si>
-    <t xml:space="preserve">BYD02 </t>
-  </si>
-  <si>
     <t xml:space="preserve">BLACK TIME GREY               </t>
   </si>
   <si>
-    <t xml:space="preserve">BGA   </t>
-  </si>
-  <si>
     <t>BLACK&amp;GRAY DUAL COLOR/APRICITY</t>
   </si>
   <si>
-    <t xml:space="preserve">BPW   </t>
-  </si>
-  <si>
     <t xml:space="preserve">BLACK/PALLAS WHITE            </t>
   </si>
   <si>
-    <t xml:space="preserve">BYD07 </t>
-  </si>
-  <si>
     <t xml:space="preserve">GLACIER BLUE                  </t>
   </si>
   <si>
@@ -104,21 +77,12 @@
     <t xml:space="preserve">GLACIER BLUE/BLACK&amp;DUAL COLOR </t>
   </si>
   <si>
-    <t xml:space="preserve">D009  </t>
-  </si>
-  <si>
     <t xml:space="preserve">MALACHITE DARKCYAN            </t>
   </si>
   <si>
-    <t xml:space="preserve">MDB   </t>
-  </si>
-  <si>
     <t xml:space="preserve">MALACHITE DARKCYAN/BLACK      </t>
   </si>
   <si>
-    <t xml:space="preserve">OBLA  </t>
-  </si>
-  <si>
     <t xml:space="preserve">OBSIDIAN BLACK                </t>
   </si>
   <si>
@@ -131,9 +95,6 @@
     <t>BYD007</t>
   </si>
   <si>
-    <t>OBSIDIAN BLACK/BLACK&amp;GRAY DUAL</t>
-  </si>
-  <si>
     <t>BYD013</t>
   </si>
   <si>
@@ -146,33 +107,18 @@
     <t xml:space="preserve">OBSIDIAN BLUE P.              </t>
   </si>
   <si>
-    <t xml:space="preserve">PLL   </t>
-  </si>
-  <si>
     <t xml:space="preserve">PALLAS WHITE                  </t>
   </si>
   <si>
-    <t xml:space="preserve">PLWB  </t>
-  </si>
-  <si>
     <t xml:space="preserve">PALLAS WHITE/BLACK            </t>
   </si>
   <si>
-    <t xml:space="preserve">BY013 </t>
-  </si>
-  <si>
     <t xml:space="preserve">SMOKE GRAY/BLACK              </t>
   </si>
   <si>
-    <t xml:space="preserve">SNWH  </t>
-  </si>
-  <si>
     <t xml:space="preserve">SNOW WHITE                    </t>
   </si>
   <si>
-    <t xml:space="preserve">SWB   </t>
-  </si>
-  <si>
     <t xml:space="preserve">SNOW WHITE/BLACK              </t>
   </si>
   <si>
@@ -182,15 +128,9 @@
     <t xml:space="preserve">SNOW WHITE/GRAVEL BEIGE       </t>
   </si>
   <si>
-    <t xml:space="preserve">BYD11 </t>
-  </si>
-  <si>
     <t>TIME GREY/BASALT BLACK+READ HA</t>
   </si>
   <si>
-    <t xml:space="preserve">TGR   </t>
-  </si>
-  <si>
     <t xml:space="preserve">TIME GREY/BLACK               </t>
   </si>
   <si>
@@ -198,6 +138,90 @@
   </si>
   <si>
     <t xml:space="preserve">TIME GREY/GRAVEL BEIGE        </t>
+  </si>
+  <si>
+    <t>TITANIUM METALIC GREY/BLACK AND BLUE</t>
+  </si>
+  <si>
+    <t>BYD017</t>
+  </si>
+  <si>
+    <t>JUNGLE GREEN/BLACK BLUE</t>
+  </si>
+  <si>
+    <t>OBSIDIAN BLACK/BLACK AND BLUE</t>
+  </si>
+  <si>
+    <t>OBSIDIAN BLACK/BLACK&amp;GREY</t>
+  </si>
+  <si>
+    <t>BYD009</t>
+  </si>
+  <si>
+    <t>TGR</t>
+  </si>
+  <si>
+    <t>BYD11</t>
+  </si>
+  <si>
+    <t>SWB</t>
+  </si>
+  <si>
+    <t>SNWH</t>
+  </si>
+  <si>
+    <t>BY013</t>
+  </si>
+  <si>
+    <t>PLWB</t>
+  </si>
+  <si>
+    <t>PLL</t>
+  </si>
+  <si>
+    <t>BYD019</t>
+  </si>
+  <si>
+    <t>OBLA</t>
+  </si>
+  <si>
+    <t>MDB</t>
+  </si>
+  <si>
+    <t>D009</t>
+  </si>
+  <si>
+    <t>BYD018</t>
+  </si>
+  <si>
+    <t>BYD07</t>
+  </si>
+  <si>
+    <t>BPW</t>
+  </si>
+  <si>
+    <t>BGA</t>
+  </si>
+  <si>
+    <t>BYD02</t>
+  </si>
+  <si>
+    <t>BYD04</t>
+  </si>
+  <si>
+    <t>BYD01</t>
+  </si>
+  <si>
+    <t>AGB</t>
+  </si>
+  <si>
+    <t>DYB07</t>
+  </si>
+  <si>
+    <t>BYD06</t>
+  </si>
+  <si>
+    <t>TIME GREY/BLACK&amp;GREY</t>
   </si>
 </sst>
 </file>
@@ -518,13 +542,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B33"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="35" customWidth="1"/>
+    <col min="2" max="2" width="37.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -532,231 +556,264 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
+        <v>64</v>
+      </c>
+      <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
         <v>4</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B4" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
         <v>6</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B5" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>62</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="B5" t="s">
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>61</v>
+      </c>
+      <c r="B7" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B8" t="s">
         <v>10</v>
       </c>
-      <c r="B6" t="s">
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>59</v>
+      </c>
+      <c r="B9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>58</v>
+      </c>
+      <c r="B10" t="s">
         <v>12</v>
       </c>
-      <c r="B7" t="s">
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B11" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>56</v>
+      </c>
+      <c r="B12" t="s">
         <v>14</v>
       </c>
-      <c r="B8" t="s">
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="B13" t="s">
         <v>16</v>
       </c>
-      <c r="B9" t="s">
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>55</v>
+      </c>
+      <c r="B14" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>54</v>
+      </c>
+      <c r="B15" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>53</v>
+      </c>
+      <c r="B16" t="s">
         <v>18</v>
       </c>
-      <c r="B10" t="s">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>52</v>
+      </c>
+      <c r="B17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
         <v>20</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B18" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
         <v>22</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="B21" t="s">
         <v>24</v>
       </c>
-      <c r="B13" t="s">
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="B22" t="s">
         <v>26</v>
       </c>
-      <c r="B14" t="s">
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>49</v>
+      </c>
+      <c r="B24" t="s">
         <v>28</v>
       </c>
-      <c r="B15" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>30</v>
-      </c>
-      <c r="B16" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>32</v>
-      </c>
-      <c r="B17" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>34</v>
-      </c>
-      <c r="B18" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>38</v>
-      </c>
-      <c r="B20" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>40</v>
-      </c>
-      <c r="B21" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>42</v>
-      </c>
-      <c r="B22" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B23" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>46</v>
-      </c>
-      <c r="B24" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>48</v>
       </c>
       <c r="B25" t="s">
-        <v>49</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B26" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B27" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>54</v>
+        <v>32</v>
       </c>
       <c r="B28" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="B29" t="s">
-        <v>57</v>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>44</v>
+      </c>
+      <c r="B30" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>43</v>
+      </c>
+      <c r="B31" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>36</v>
+      </c>
+      <c r="B32" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>